<commit_message>
updated dates on supplemtn planner
</commit_message>
<xml_diff>
--- a/public/downloads/LOE Supplement Planner_V1.1.xlsx
+++ b/public/downloads/LOE Supplement Planner_V1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katy/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katy/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526B74CB-82E2-A343-B905-EAB2D86D7453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713C3258-F98A-CA42-8163-366D235D2446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LOE Supplement Planner" sheetId="1" r:id="rId1"/>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="55">
   <si>
     <t>PI Name</t>
   </si>
@@ -268,6 +268,57 @@
   </si>
   <si>
     <t>End Date</t>
+  </si>
+  <si>
+    <t>Jul-26</t>
+  </si>
+  <si>
+    <t>Aug-26</t>
+  </si>
+  <si>
+    <t>Sep-26</t>
+  </si>
+  <si>
+    <t>Oct-26</t>
+  </si>
+  <si>
+    <t>Nov-26</t>
+  </si>
+  <si>
+    <t>Dec-26</t>
+  </si>
+  <si>
+    <t>Jan-27</t>
+  </si>
+  <si>
+    <t>Feb-27</t>
+  </si>
+  <si>
+    <t>Mar-27</t>
+  </si>
+  <si>
+    <t>Apr-27</t>
+  </si>
+  <si>
+    <t>May-27</t>
+  </si>
+  <si>
+    <t>Jun-27</t>
+  </si>
+  <si>
+    <t>Input Guidance
+• Enter PI compensation inputs before entering LOE distributions.
+• Monthly FTE cells are editable and default to 100%.
+• Update only months where appointment/FTE changes.
+• Yellow indicates FTE below 100%; red indicates FTE above 100%.
+• Monthly calculations use each month’s FTE directly.
+• Monthly LOE totals should equal 100%.
+Summary Guidance
+• Average values are calculated automatically from the monthly FTE row.
+• “Without Supplement” excludes supplement compensation from calculations.
+• “With Supplement” includes supplement compensation and scaling logic.
+• Dollar values calculate automatically from salary, FTE, supplement logic, and LOE percentages.
+• Changes to monthly FTE values automatically update monthly compensation calculations.</t>
   </si>
 </sst>
 </file>
@@ -1228,6 +1279,95 @@
     <xf numFmtId="44" fontId="4" fillId="5" borderId="59" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="44" fontId="4" fillId="5" borderId="60" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="10" fontId="5" fillId="7" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1256,8 +1396,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -1322,93 +1460,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1928,39 +1979,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="28" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="84" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
       <c r="E1" s="34"/>
       <c r="F1" s="34"/>
       <c r="G1" s="34"/>
-      <c r="H1" s="67" t="s">
+      <c r="H1" s="100" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
-      <c r="V1" s="67"/>
-      <c r="W1" s="67"/>
-      <c r="X1" s="67"/>
-      <c r="Y1" s="67"/>
-      <c r="Z1" s="67"/>
-      <c r="AA1" s="67"/>
-      <c r="AB1" s="67"/>
-      <c r="AC1" s="67"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="100"/>
+      <c r="N1" s="100"/>
+      <c r="O1" s="100"/>
+      <c r="P1" s="100"/>
+      <c r="Q1" s="100"/>
+      <c r="R1" s="100"/>
+      <c r="S1" s="100"/>
+      <c r="T1" s="100"/>
+      <c r="U1" s="100"/>
+      <c r="V1" s="100"/>
+      <c r="W1" s="100"/>
+      <c r="X1" s="100"/>
+      <c r="Y1" s="100"/>
+      <c r="Z1" s="100"/>
+      <c r="AA1" s="100"/>
+      <c r="AB1" s="100"/>
+      <c r="AC1" s="100"/>
       <c r="AD1" s="34"/>
       <c r="AE1" s="34"/>
       <c r="AF1" s="34"/>
@@ -1970,34 +2021,36 @@
       <c r="A2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="72"/>
+      <c r="B2" s="102"/>
+      <c r="C2" s="102"/>
+      <c r="D2" s="103"/>
       <c r="E2" s="37"/>
       <c r="F2" s="37"/>
       <c r="G2" s="37"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="63"/>
-      <c r="M2" s="63"/>
-      <c r="N2" s="63"/>
-      <c r="O2" s="63"/>
-      <c r="P2" s="63"/>
-      <c r="Q2" s="63"/>
-      <c r="R2" s="63"/>
-      <c r="S2" s="63"/>
-      <c r="T2" s="63"/>
-      <c r="U2" s="63"/>
-      <c r="V2" s="63"/>
-      <c r="W2" s="63"/>
-      <c r="X2" s="63"/>
-      <c r="Y2" s="63"/>
-      <c r="Z2" s="63"/>
-      <c r="AA2" s="63"/>
-      <c r="AB2" s="63"/>
-      <c r="AC2" s="63"/>
+      <c r="H2" s="96" t="s">
+        <v>54</v>
+      </c>
+      <c r="I2" s="96"/>
+      <c r="J2" s="96"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="96"/>
+      <c r="M2" s="96"/>
+      <c r="N2" s="96"/>
+      <c r="O2" s="96"/>
+      <c r="P2" s="96"/>
+      <c r="Q2" s="96"/>
+      <c r="R2" s="96"/>
+      <c r="S2" s="96"/>
+      <c r="T2" s="96"/>
+      <c r="U2" s="96"/>
+      <c r="V2" s="96"/>
+      <c r="W2" s="96"/>
+      <c r="X2" s="96"/>
+      <c r="Y2" s="96"/>
+      <c r="Z2" s="96"/>
+      <c r="AA2" s="96"/>
+      <c r="AB2" s="96"/>
+      <c r="AC2" s="96"/>
       <c r="AD2" s="37"/>
       <c r="AE2" s="37"/>
       <c r="AF2" s="37"/>
@@ -2007,34 +2060,34 @@
       <c r="A3" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="74"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="105"/>
       <c r="E3" s="37"/>
       <c r="F3" s="37"/>
       <c r="G3" s="37"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="64"/>
-      <c r="M3" s="64"/>
-      <c r="N3" s="64"/>
-      <c r="O3" s="64"/>
-      <c r="P3" s="64"/>
-      <c r="Q3" s="64"/>
-      <c r="R3" s="64"/>
-      <c r="S3" s="64"/>
-      <c r="T3" s="64"/>
-      <c r="U3" s="64"/>
-      <c r="V3" s="64"/>
-      <c r="W3" s="64"/>
-      <c r="X3" s="64"/>
-      <c r="Y3" s="64"/>
-      <c r="Z3" s="64"/>
-      <c r="AA3" s="64"/>
-      <c r="AB3" s="64"/>
-      <c r="AC3" s="64"/>
+      <c r="H3" s="97"/>
+      <c r="I3" s="97"/>
+      <c r="J3" s="97"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
+      <c r="M3" s="97"/>
+      <c r="N3" s="97"/>
+      <c r="O3" s="97"/>
+      <c r="P3" s="97"/>
+      <c r="Q3" s="97"/>
+      <c r="R3" s="97"/>
+      <c r="S3" s="97"/>
+      <c r="T3" s="97"/>
+      <c r="U3" s="97"/>
+      <c r="V3" s="97"/>
+      <c r="W3" s="97"/>
+      <c r="X3" s="97"/>
+      <c r="Y3" s="97"/>
+      <c r="Z3" s="97"/>
+      <c r="AA3" s="97"/>
+      <c r="AB3" s="97"/>
+      <c r="AC3" s="97"/>
       <c r="AD3" s="37"/>
       <c r="AE3" s="37"/>
       <c r="AF3" s="37"/>
@@ -2044,34 +2097,34 @@
       <c r="A4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="76"/>
+      <c r="B4" s="106"/>
+      <c r="C4" s="106"/>
+      <c r="D4" s="107"/>
       <c r="E4" s="37"/>
       <c r="F4" s="37"/>
       <c r="G4" s="37"/>
-      <c r="H4" s="64"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="64"/>
-      <c r="M4" s="64"/>
-      <c r="N4" s="64"/>
-      <c r="O4" s="64"/>
-      <c r="P4" s="64"/>
-      <c r="Q4" s="64"/>
-      <c r="R4" s="64"/>
-      <c r="S4" s="64"/>
-      <c r="T4" s="64"/>
-      <c r="U4" s="64"/>
-      <c r="V4" s="64"/>
-      <c r="W4" s="64"/>
-      <c r="X4" s="64"/>
-      <c r="Y4" s="64"/>
-      <c r="Z4" s="64"/>
-      <c r="AA4" s="64"/>
-      <c r="AB4" s="64"/>
-      <c r="AC4" s="64"/>
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="97"/>
+      <c r="K4" s="97"/>
+      <c r="L4" s="97"/>
+      <c r="M4" s="97"/>
+      <c r="N4" s="97"/>
+      <c r="O4" s="97"/>
+      <c r="P4" s="97"/>
+      <c r="Q4" s="97"/>
+      <c r="R4" s="97"/>
+      <c r="S4" s="97"/>
+      <c r="T4" s="97"/>
+      <c r="U4" s="97"/>
+      <c r="V4" s="97"/>
+      <c r="W4" s="97"/>
+      <c r="X4" s="97"/>
+      <c r="Y4" s="97"/>
+      <c r="Z4" s="97"/>
+      <c r="AA4" s="97"/>
+      <c r="AB4" s="97"/>
+      <c r="AC4" s="97"/>
       <c r="AD4" s="37"/>
       <c r="AE4" s="37"/>
       <c r="AF4" s="37"/>
@@ -2081,37 +2134,37 @@
       <c r="A5" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="77">
+      <c r="B5" s="108">
         <f>($B$4/12)*$B$10</f>
         <v>0</v>
       </c>
-      <c r="C5" s="77"/>
-      <c r="D5" s="78"/>
+      <c r="C5" s="108"/>
+      <c r="D5" s="109"/>
       <c r="E5" s="37"/>
       <c r="F5" s="37"/>
       <c r="G5" s="37"/>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="64"/>
-      <c r="L5" s="64"/>
-      <c r="M5" s="64"/>
-      <c r="N5" s="64"/>
-      <c r="O5" s="64"/>
-      <c r="P5" s="64"/>
-      <c r="Q5" s="64"/>
-      <c r="R5" s="64"/>
-      <c r="S5" s="64"/>
-      <c r="T5" s="64"/>
-      <c r="U5" s="64"/>
-      <c r="V5" s="64"/>
-      <c r="W5" s="64"/>
-      <c r="X5" s="64"/>
-      <c r="Y5" s="64"/>
-      <c r="Z5" s="64"/>
-      <c r="AA5" s="64"/>
-      <c r="AB5" s="64"/>
-      <c r="AC5" s="64"/>
+      <c r="H5" s="97"/>
+      <c r="I5" s="97"/>
+      <c r="J5" s="97"/>
+      <c r="K5" s="97"/>
+      <c r="L5" s="97"/>
+      <c r="M5" s="97"/>
+      <c r="N5" s="97"/>
+      <c r="O5" s="97"/>
+      <c r="P5" s="97"/>
+      <c r="Q5" s="97"/>
+      <c r="R5" s="97"/>
+      <c r="S5" s="97"/>
+      <c r="T5" s="97"/>
+      <c r="U5" s="97"/>
+      <c r="V5" s="97"/>
+      <c r="W5" s="97"/>
+      <c r="X5" s="97"/>
+      <c r="Y5" s="97"/>
+      <c r="Z5" s="97"/>
+      <c r="AA5" s="97"/>
+      <c r="AB5" s="97"/>
+      <c r="AC5" s="97"/>
       <c r="AD5" s="37"/>
       <c r="AE5" s="37"/>
       <c r="AF5" s="37"/>
@@ -2121,34 +2174,34 @@
       <c r="A6" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="76"/>
+      <c r="B6" s="106"/>
+      <c r="C6" s="106"/>
+      <c r="D6" s="107"/>
       <c r="E6" s="37"/>
       <c r="F6" s="37"/>
       <c r="G6" s="37"/>
-      <c r="H6" s="64"/>
-      <c r="I6" s="64"/>
-      <c r="J6" s="64"/>
-      <c r="K6" s="64"/>
-      <c r="L6" s="64"/>
-      <c r="M6" s="64"/>
-      <c r="N6" s="64"/>
-      <c r="O6" s="64"/>
-      <c r="P6" s="64"/>
-      <c r="Q6" s="64"/>
-      <c r="R6" s="64"/>
-      <c r="S6" s="64"/>
-      <c r="T6" s="64"/>
-      <c r="U6" s="64"/>
-      <c r="V6" s="64"/>
-      <c r="W6" s="64"/>
-      <c r="X6" s="64"/>
-      <c r="Y6" s="64"/>
-      <c r="Z6" s="64"/>
-      <c r="AA6" s="64"/>
-      <c r="AB6" s="64"/>
-      <c r="AC6" s="64"/>
+      <c r="H6" s="97"/>
+      <c r="I6" s="97"/>
+      <c r="J6" s="97"/>
+      <c r="K6" s="97"/>
+      <c r="L6" s="97"/>
+      <c r="M6" s="97"/>
+      <c r="N6" s="97"/>
+      <c r="O6" s="97"/>
+      <c r="P6" s="97"/>
+      <c r="Q6" s="97"/>
+      <c r="R6" s="97"/>
+      <c r="S6" s="97"/>
+      <c r="T6" s="97"/>
+      <c r="U6" s="97"/>
+      <c r="V6" s="97"/>
+      <c r="W6" s="97"/>
+      <c r="X6" s="97"/>
+      <c r="Y6" s="97"/>
+      <c r="Z6" s="97"/>
+      <c r="AA6" s="97"/>
+      <c r="AB6" s="97"/>
+      <c r="AC6" s="97"/>
       <c r="AD6" s="37"/>
       <c r="AE6" s="37"/>
       <c r="AF6" s="37"/>
@@ -2158,37 +2211,37 @@
       <c r="A7" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="79">
+      <c r="B7" s="110">
         <f>IF($B$11="Yes",($B$6/12)*$B$10,$B$6/12)</f>
         <v>0</v>
       </c>
-      <c r="C7" s="79"/>
-      <c r="D7" s="80"/>
+      <c r="C7" s="110"/>
+      <c r="D7" s="111"/>
       <c r="E7" s="37"/>
       <c r="F7" s="37"/>
       <c r="G7" s="37"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
-      <c r="J7" s="64"/>
-      <c r="K7" s="64"/>
-      <c r="L7" s="64"/>
-      <c r="M7" s="64"/>
-      <c r="N7" s="64"/>
-      <c r="O7" s="64"/>
-      <c r="P7" s="64"/>
-      <c r="Q7" s="64"/>
-      <c r="R7" s="64"/>
-      <c r="S7" s="64"/>
-      <c r="T7" s="64"/>
-      <c r="U7" s="64"/>
-      <c r="V7" s="64"/>
-      <c r="W7" s="64"/>
-      <c r="X7" s="64"/>
-      <c r="Y7" s="64"/>
-      <c r="Z7" s="64"/>
-      <c r="AA7" s="64"/>
-      <c r="AB7" s="64"/>
-      <c r="AC7" s="64"/>
+      <c r="H7" s="97"/>
+      <c r="I7" s="97"/>
+      <c r="J7" s="97"/>
+      <c r="K7" s="97"/>
+      <c r="L7" s="97"/>
+      <c r="M7" s="97"/>
+      <c r="N7" s="97"/>
+      <c r="O7" s="97"/>
+      <c r="P7" s="97"/>
+      <c r="Q7" s="97"/>
+      <c r="R7" s="97"/>
+      <c r="S7" s="97"/>
+      <c r="T7" s="97"/>
+      <c r="U7" s="97"/>
+      <c r="V7" s="97"/>
+      <c r="W7" s="97"/>
+      <c r="X7" s="97"/>
+      <c r="Y7" s="97"/>
+      <c r="Z7" s="97"/>
+      <c r="AA7" s="97"/>
+      <c r="AB7" s="97"/>
+      <c r="AC7" s="97"/>
       <c r="AD7" s="37"/>
       <c r="AE7" s="37"/>
       <c r="AF7" s="37"/>
@@ -2198,34 +2251,34 @@
       <c r="A8" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="81"/>
-      <c r="C8" s="81"/>
-      <c r="D8" s="82"/>
+      <c r="B8" s="112"/>
+      <c r="C8" s="112"/>
+      <c r="D8" s="113"/>
       <c r="E8" s="37"/>
       <c r="F8" s="37"/>
       <c r="G8" s="37"/>
-      <c r="H8" s="64"/>
-      <c r="I8" s="64"/>
-      <c r="J8" s="64"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="64"/>
-      <c r="M8" s="64"/>
-      <c r="N8" s="64"/>
-      <c r="O8" s="64"/>
-      <c r="P8" s="64"/>
-      <c r="Q8" s="64"/>
-      <c r="R8" s="64"/>
-      <c r="S8" s="64"/>
-      <c r="T8" s="64"/>
-      <c r="U8" s="64"/>
-      <c r="V8" s="64"/>
-      <c r="W8" s="64"/>
-      <c r="X8" s="64"/>
-      <c r="Y8" s="64"/>
-      <c r="Z8" s="64"/>
-      <c r="AA8" s="64"/>
-      <c r="AB8" s="64"/>
-      <c r="AC8" s="64"/>
+      <c r="H8" s="97"/>
+      <c r="I8" s="97"/>
+      <c r="J8" s="97"/>
+      <c r="K8" s="97"/>
+      <c r="L8" s="97"/>
+      <c r="M8" s="97"/>
+      <c r="N8" s="97"/>
+      <c r="O8" s="97"/>
+      <c r="P8" s="97"/>
+      <c r="Q8" s="97"/>
+      <c r="R8" s="97"/>
+      <c r="S8" s="97"/>
+      <c r="T8" s="97"/>
+      <c r="U8" s="97"/>
+      <c r="V8" s="97"/>
+      <c r="W8" s="97"/>
+      <c r="X8" s="97"/>
+      <c r="Y8" s="97"/>
+      <c r="Z8" s="97"/>
+      <c r="AA8" s="97"/>
+      <c r="AB8" s="97"/>
+      <c r="AC8" s="97"/>
       <c r="AD8" s="37"/>
       <c r="AE8" s="37"/>
       <c r="AF8" s="37"/>
@@ -2235,34 +2288,34 @@
       <c r="A9" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="83"/>
-      <c r="C9" s="83"/>
-      <c r="D9" s="84"/>
+      <c r="B9" s="114"/>
+      <c r="C9" s="114"/>
+      <c r="D9" s="115"/>
       <c r="E9" s="37"/>
       <c r="F9" s="37"/>
       <c r="G9" s="37"/>
-      <c r="H9" s="64"/>
-      <c r="I9" s="64"/>
-      <c r="J9" s="64"/>
-      <c r="K9" s="64"/>
-      <c r="L9" s="64"/>
-      <c r="M9" s="64"/>
-      <c r="N9" s="64"/>
-      <c r="O9" s="64"/>
-      <c r="P9" s="64"/>
-      <c r="Q9" s="64"/>
-      <c r="R9" s="64"/>
-      <c r="S9" s="64"/>
-      <c r="T9" s="64"/>
-      <c r="U9" s="64"/>
-      <c r="V9" s="64"/>
-      <c r="W9" s="64"/>
-      <c r="X9" s="64"/>
-      <c r="Y9" s="64"/>
-      <c r="Z9" s="64"/>
-      <c r="AA9" s="64"/>
-      <c r="AB9" s="64"/>
-      <c r="AC9" s="64"/>
+      <c r="H9" s="97"/>
+      <c r="I9" s="97"/>
+      <c r="J9" s="97"/>
+      <c r="K9" s="97"/>
+      <c r="L9" s="97"/>
+      <c r="M9" s="97"/>
+      <c r="N9" s="97"/>
+      <c r="O9" s="97"/>
+      <c r="P9" s="97"/>
+      <c r="Q9" s="97"/>
+      <c r="R9" s="97"/>
+      <c r="S9" s="97"/>
+      <c r="T9" s="97"/>
+      <c r="U9" s="97"/>
+      <c r="V9" s="97"/>
+      <c r="W9" s="97"/>
+      <c r="X9" s="97"/>
+      <c r="Y9" s="97"/>
+      <c r="Z9" s="97"/>
+      <c r="AA9" s="97"/>
+      <c r="AB9" s="97"/>
+      <c r="AC9" s="97"/>
       <c r="AD9" s="37"/>
       <c r="AE9" s="37"/>
       <c r="AF9" s="37"/>
@@ -2272,34 +2325,34 @@
       <c r="A10" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="110"/>
-      <c r="C10" s="110"/>
-      <c r="D10" s="111"/>
+      <c r="B10" s="65"/>
+      <c r="C10" s="65"/>
+      <c r="D10" s="66"/>
       <c r="E10" s="37"/>
       <c r="F10" s="37"/>
       <c r="G10" s="37"/>
-      <c r="H10" s="64"/>
-      <c r="I10" s="64"/>
-      <c r="J10" s="64"/>
-      <c r="K10" s="64"/>
-      <c r="L10" s="64"/>
-      <c r="M10" s="64"/>
-      <c r="N10" s="64"/>
-      <c r="O10" s="64"/>
-      <c r="P10" s="64"/>
-      <c r="Q10" s="64"/>
-      <c r="R10" s="64"/>
-      <c r="S10" s="64"/>
-      <c r="T10" s="64"/>
-      <c r="U10" s="64"/>
-      <c r="V10" s="64"/>
-      <c r="W10" s="64"/>
-      <c r="X10" s="64"/>
-      <c r="Y10" s="64"/>
-      <c r="Z10" s="64"/>
-      <c r="AA10" s="64"/>
-      <c r="AB10" s="64"/>
-      <c r="AC10" s="64"/>
+      <c r="H10" s="97"/>
+      <c r="I10" s="97"/>
+      <c r="J10" s="97"/>
+      <c r="K10" s="97"/>
+      <c r="L10" s="97"/>
+      <c r="M10" s="97"/>
+      <c r="N10" s="97"/>
+      <c r="O10" s="97"/>
+      <c r="P10" s="97"/>
+      <c r="Q10" s="97"/>
+      <c r="R10" s="97"/>
+      <c r="S10" s="97"/>
+      <c r="T10" s="97"/>
+      <c r="U10" s="97"/>
+      <c r="V10" s="97"/>
+      <c r="W10" s="97"/>
+      <c r="X10" s="97"/>
+      <c r="Y10" s="97"/>
+      <c r="Z10" s="97"/>
+      <c r="AA10" s="97"/>
+      <c r="AB10" s="97"/>
+      <c r="AC10" s="97"/>
       <c r="AD10" s="37"/>
       <c r="AE10" s="37"/>
       <c r="AF10" s="37"/>
@@ -2309,34 +2362,34 @@
       <c r="A11" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="61"/>
+      <c r="B11" s="93"/>
+      <c r="C11" s="93"/>
+      <c r="D11" s="94"/>
       <c r="E11" s="37"/>
       <c r="F11" s="37"/>
       <c r="G11" s="37"/>
-      <c r="H11" s="64"/>
-      <c r="I11" s="64"/>
-      <c r="J11" s="64"/>
-      <c r="K11" s="64"/>
-      <c r="L11" s="64"/>
-      <c r="M11" s="64"/>
-      <c r="N11" s="64"/>
-      <c r="O11" s="64"/>
-      <c r="P11" s="64"/>
-      <c r="Q11" s="64"/>
-      <c r="R11" s="64"/>
-      <c r="S11" s="64"/>
-      <c r="T11" s="64"/>
-      <c r="U11" s="64"/>
-      <c r="V11" s="64"/>
-      <c r="W11" s="64"/>
-      <c r="X11" s="64"/>
-      <c r="Y11" s="64"/>
-      <c r="Z11" s="64"/>
-      <c r="AA11" s="64"/>
-      <c r="AB11" s="64"/>
-      <c r="AC11" s="64"/>
+      <c r="H11" s="97"/>
+      <c r="I11" s="97"/>
+      <c r="J11" s="97"/>
+      <c r="K11" s="97"/>
+      <c r="L11" s="97"/>
+      <c r="M11" s="97"/>
+      <c r="N11" s="97"/>
+      <c r="O11" s="97"/>
+      <c r="P11" s="97"/>
+      <c r="Q11" s="97"/>
+      <c r="R11" s="97"/>
+      <c r="S11" s="97"/>
+      <c r="T11" s="97"/>
+      <c r="U11" s="97"/>
+      <c r="V11" s="97"/>
+      <c r="W11" s="97"/>
+      <c r="X11" s="97"/>
+      <c r="Y11" s="97"/>
+      <c r="Z11" s="97"/>
+      <c r="AA11" s="97"/>
+      <c r="AB11" s="97"/>
+      <c r="AC11" s="97"/>
       <c r="AD11" s="37"/>
       <c r="AE11" s="37"/>
       <c r="AF11" s="37"/>
@@ -2346,37 +2399,37 @@
       <c r="A12" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="85">
+      <c r="B12" s="116">
         <f>$B$5+$B$7</f>
         <v>0</v>
       </c>
-      <c r="C12" s="85"/>
-      <c r="D12" s="86"/>
+      <c r="C12" s="116"/>
+      <c r="D12" s="117"/>
       <c r="E12" s="37"/>
       <c r="F12" s="37"/>
       <c r="G12" s="37"/>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
-      <c r="J12" s="64"/>
-      <c r="K12" s="64"/>
-      <c r="L12" s="64"/>
-      <c r="M12" s="64"/>
-      <c r="N12" s="64"/>
-      <c r="O12" s="64"/>
-      <c r="P12" s="64"/>
-      <c r="Q12" s="64"/>
-      <c r="R12" s="64"/>
-      <c r="S12" s="64"/>
-      <c r="T12" s="64"/>
-      <c r="U12" s="64"/>
-      <c r="V12" s="64"/>
-      <c r="W12" s="64"/>
-      <c r="X12" s="64"/>
-      <c r="Y12" s="64"/>
-      <c r="Z12" s="64"/>
-      <c r="AA12" s="64"/>
-      <c r="AB12" s="64"/>
-      <c r="AC12" s="64"/>
+      <c r="H12" s="97"/>
+      <c r="I12" s="97"/>
+      <c r="J12" s="97"/>
+      <c r="K12" s="97"/>
+      <c r="L12" s="97"/>
+      <c r="M12" s="97"/>
+      <c r="N12" s="97"/>
+      <c r="O12" s="97"/>
+      <c r="P12" s="97"/>
+      <c r="Q12" s="97"/>
+      <c r="R12" s="97"/>
+      <c r="S12" s="97"/>
+      <c r="T12" s="97"/>
+      <c r="U12" s="97"/>
+      <c r="V12" s="97"/>
+      <c r="W12" s="97"/>
+      <c r="X12" s="97"/>
+      <c r="Y12" s="97"/>
+      <c r="Z12" s="97"/>
+      <c r="AA12" s="97"/>
+      <c r="AB12" s="97"/>
+      <c r="AC12" s="97"/>
       <c r="AD12" s="37"/>
       <c r="AE12" s="37"/>
       <c r="AF12" s="37"/>
@@ -2386,197 +2439,197 @@
       <c r="A13" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="62">
+      <c r="B13" s="95">
         <f>$B$12*(1+$B$8)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="62"/>
-      <c r="D13" s="62"/>
+      <c r="C13" s="95"/>
+      <c r="D13" s="95"/>
       <c r="E13" s="37"/>
       <c r="F13" s="37"/>
       <c r="G13" s="37"/>
-      <c r="H13" s="64"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="64"/>
-      <c r="K13" s="64"/>
-      <c r="L13" s="64"/>
-      <c r="M13" s="64"/>
-      <c r="N13" s="64"/>
-      <c r="O13" s="64"/>
-      <c r="P13" s="64"/>
-      <c r="Q13" s="64"/>
-      <c r="R13" s="64"/>
-      <c r="S13" s="64"/>
-      <c r="T13" s="64"/>
-      <c r="U13" s="64"/>
-      <c r="V13" s="64"/>
-      <c r="W13" s="64"/>
-      <c r="X13" s="64"/>
-      <c r="Y13" s="64"/>
-      <c r="Z13" s="64"/>
-      <c r="AA13" s="64"/>
-      <c r="AB13" s="64"/>
-      <c r="AC13" s="64"/>
+      <c r="H13" s="97"/>
+      <c r="I13" s="97"/>
+      <c r="J13" s="97"/>
+      <c r="K13" s="97"/>
+      <c r="L13" s="97"/>
+      <c r="M13" s="97"/>
+      <c r="N13" s="97"/>
+      <c r="O13" s="97"/>
+      <c r="P13" s="97"/>
+      <c r="Q13" s="97"/>
+      <c r="R13" s="97"/>
+      <c r="S13" s="97"/>
+      <c r="T13" s="97"/>
+      <c r="U13" s="97"/>
+      <c r="V13" s="97"/>
+      <c r="W13" s="97"/>
+      <c r="X13" s="97"/>
+      <c r="Y13" s="97"/>
+      <c r="Z13" s="97"/>
+      <c r="AA13" s="97"/>
+      <c r="AB13" s="97"/>
+      <c r="AC13" s="97"/>
       <c r="AD13" s="37"/>
       <c r="AE13" s="37"/>
       <c r="AF13" s="37"/>
       <c r="AG13" s="38"/>
     </row>
     <row r="14" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="95"/>
-      <c r="B14" s="96"/>
-      <c r="C14" s="96"/>
-      <c r="D14" s="96"/>
-      <c r="E14" s="96"/>
-      <c r="F14" s="96"/>
-      <c r="G14" s="96"/>
-      <c r="H14" s="96"/>
-      <c r="I14" s="96"/>
-      <c r="J14" s="96"/>
-      <c r="K14" s="96"/>
-      <c r="L14" s="96"/>
-      <c r="M14" s="96"/>
-      <c r="N14" s="96"/>
-      <c r="O14" s="96"/>
-      <c r="P14" s="96"/>
-      <c r="Q14" s="96"/>
-      <c r="R14" s="96"/>
-      <c r="S14" s="96"/>
-      <c r="T14" s="96"/>
-      <c r="U14" s="96"/>
-      <c r="V14" s="96"/>
-      <c r="W14" s="96"/>
-      <c r="X14" s="96"/>
-      <c r="Y14" s="96"/>
-      <c r="Z14" s="96"/>
-      <c r="AA14" s="96"/>
-      <c r="AB14" s="96"/>
-      <c r="AC14" s="96"/>
-      <c r="AD14" s="96"/>
-      <c r="AE14" s="96"/>
-      <c r="AF14" s="96"/>
-      <c r="AG14" s="97"/>
+      <c r="A14" s="90"/>
+      <c r="B14" s="91"/>
+      <c r="C14" s="91"/>
+      <c r="D14" s="91"/>
+      <c r="E14" s="91"/>
+      <c r="F14" s="91"/>
+      <c r="G14" s="91"/>
+      <c r="H14" s="91"/>
+      <c r="I14" s="91"/>
+      <c r="J14" s="91"/>
+      <c r="K14" s="91"/>
+      <c r="L14" s="91"/>
+      <c r="M14" s="91"/>
+      <c r="N14" s="91"/>
+      <c r="O14" s="91"/>
+      <c r="P14" s="91"/>
+      <c r="Q14" s="91"/>
+      <c r="R14" s="91"/>
+      <c r="S14" s="91"/>
+      <c r="T14" s="91"/>
+      <c r="U14" s="91"/>
+      <c r="V14" s="91"/>
+      <c r="W14" s="91"/>
+      <c r="X14" s="91"/>
+      <c r="Y14" s="91"/>
+      <c r="Z14" s="91"/>
+      <c r="AA14" s="91"/>
+      <c r="AB14" s="91"/>
+      <c r="AC14" s="91"/>
+      <c r="AD14" s="91"/>
+      <c r="AE14" s="91"/>
+      <c r="AF14" s="91"/>
+      <c r="AG14" s="92"/>
     </row>
     <row r="15" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="68" t="s">
+      <c r="A15" s="86" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="69"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="69"/>
-      <c r="E15" s="91"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="69"/>
-      <c r="H15" s="69"/>
-      <c r="I15" s="69"/>
-      <c r="J15" s="69"/>
-      <c r="K15" s="69"/>
-      <c r="L15" s="69"/>
-      <c r="M15" s="69"/>
-      <c r="N15" s="69"/>
-      <c r="O15" s="69"/>
-      <c r="P15" s="69"/>
-      <c r="Q15" s="69"/>
-      <c r="R15" s="69"/>
-      <c r="S15" s="69"/>
-      <c r="T15" s="69"/>
-      <c r="U15" s="69"/>
-      <c r="V15" s="69"/>
-      <c r="W15" s="69"/>
-      <c r="X15" s="69"/>
-      <c r="Y15" s="69"/>
-      <c r="Z15" s="69"/>
-      <c r="AA15" s="69"/>
-      <c r="AB15" s="69"/>
-      <c r="AC15" s="69"/>
-      <c r="AD15" s="69"/>
-      <c r="AE15" s="69"/>
-      <c r="AF15" s="69"/>
-      <c r="AG15" s="92"/>
+      <c r="B15" s="87"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="87"/>
+      <c r="E15" s="88"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="87"/>
+      <c r="H15" s="87"/>
+      <c r="I15" s="87"/>
+      <c r="J15" s="87"/>
+      <c r="K15" s="87"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="87"/>
+      <c r="N15" s="87"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="87"/>
+      <c r="Q15" s="87"/>
+      <c r="R15" s="87"/>
+      <c r="S15" s="87"/>
+      <c r="T15" s="87"/>
+      <c r="U15" s="87"/>
+      <c r="V15" s="87"/>
+      <c r="W15" s="87"/>
+      <c r="X15" s="87"/>
+      <c r="Y15" s="87"/>
+      <c r="Z15" s="87"/>
+      <c r="AA15" s="87"/>
+      <c r="AB15" s="87"/>
+      <c r="AC15" s="87"/>
+      <c r="AD15" s="87"/>
+      <c r="AE15" s="87"/>
+      <c r="AF15" s="87"/>
+      <c r="AG15" s="89"/>
     </row>
     <row r="16" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="112" t="s">
+      <c r="A16" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="114" t="s">
+      <c r="B16" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="114" t="s">
+      <c r="C16" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="114" t="s">
+      <c r="D16" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="119" t="s">
+      <c r="E16" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="F16" s="93" t="s">
-        <v>11</v>
-      </c>
-      <c r="G16" s="94"/>
-      <c r="H16" s="93" t="s">
-        <v>12</v>
-      </c>
-      <c r="I16" s="94"/>
-      <c r="J16" s="93" t="s">
-        <v>13</v>
-      </c>
-      <c r="K16" s="94"/>
-      <c r="L16" s="93" t="s">
-        <v>14</v>
-      </c>
-      <c r="M16" s="94"/>
-      <c r="N16" s="93" t="s">
-        <v>15</v>
-      </c>
-      <c r="O16" s="94"/>
-      <c r="P16" s="93" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q16" s="94"/>
-      <c r="R16" s="93" t="s">
-        <v>17</v>
-      </c>
-      <c r="S16" s="94"/>
-      <c r="T16" s="93" t="s">
-        <v>18</v>
-      </c>
-      <c r="U16" s="94"/>
-      <c r="V16" s="93" t="s">
-        <v>19</v>
-      </c>
-      <c r="W16" s="94"/>
-      <c r="X16" s="93" t="s">
-        <v>20</v>
-      </c>
-      <c r="Y16" s="94"/>
-      <c r="Z16" s="93" t="s">
-        <v>21</v>
-      </c>
-      <c r="AA16" s="94"/>
-      <c r="AB16" s="93" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC16" s="94"/>
-      <c r="AD16" s="98" t="s">
+      <c r="F16" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="G16" s="63"/>
+      <c r="H16" s="62" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" s="63"/>
+      <c r="J16" s="62" t="s">
+        <v>44</v>
+      </c>
+      <c r="K16" s="63"/>
+      <c r="L16" s="62" t="s">
+        <v>45</v>
+      </c>
+      <c r="M16" s="63"/>
+      <c r="N16" s="62" t="s">
+        <v>46</v>
+      </c>
+      <c r="O16" s="63"/>
+      <c r="P16" s="62" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q16" s="63"/>
+      <c r="R16" s="62" t="s">
+        <v>48</v>
+      </c>
+      <c r="S16" s="63"/>
+      <c r="T16" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="U16" s="63"/>
+      <c r="V16" s="62" t="s">
+        <v>50</v>
+      </c>
+      <c r="W16" s="63"/>
+      <c r="X16" s="62" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y16" s="63"/>
+      <c r="Z16" s="62" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA16" s="63"/>
+      <c r="AB16" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC16" s="63"/>
+      <c r="AD16" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="AE16" s="98" t="s">
+      <c r="AE16" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="AF16" s="98" t="s">
+      <c r="AF16" s="75" t="s">
         <v>25</v>
       </c>
-      <c r="AG16" s="108" t="s">
+      <c r="AG16" s="60" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:33" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="118"/>
-      <c r="B17" s="115"/>
-      <c r="C17" s="115"/>
-      <c r="D17" s="115"/>
-      <c r="E17" s="117"/>
+      <c r="A17" s="73"/>
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="70"/>
+      <c r="E17" s="72"/>
       <c r="F17" s="13" t="s">
         <v>32</v>
       </c>
@@ -2649,10 +2702,10 @@
       <c r="AC17" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="AD17" s="99"/>
-      <c r="AE17" s="99"/>
-      <c r="AF17" s="99"/>
-      <c r="AG17" s="107"/>
+      <c r="AD17" s="76"/>
+      <c r="AE17" s="76"/>
+      <c r="AF17" s="76"/>
+      <c r="AG17" s="61"/>
     </row>
     <row r="18" spans="1:33" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="44"/>
@@ -3900,13 +3953,13 @@
       </c>
     </row>
     <row r="33" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="87" t="s">
+      <c r="A33" s="118" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="88"/>
-      <c r="C33" s="88"/>
-      <c r="D33" s="88"/>
-      <c r="E33" s="88"/>
+      <c r="B33" s="119"/>
+      <c r="C33" s="119"/>
+      <c r="D33" s="119"/>
+      <c r="E33" s="119"/>
       <c r="F33" s="15">
         <f>SUM(F18:F32)</f>
         <v>0</v>
@@ -4021,195 +4074,195 @@
       </c>
     </row>
     <row r="34" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="100"/>
-      <c r="B34" s="101"/>
-      <c r="C34" s="101"/>
-      <c r="D34" s="101"/>
-      <c r="E34" s="101"/>
-      <c r="F34" s="102"/>
-      <c r="G34" s="102"/>
-      <c r="H34" s="102"/>
-      <c r="I34" s="102"/>
-      <c r="J34" s="102"/>
-      <c r="K34" s="102"/>
-      <c r="L34" s="102"/>
-      <c r="M34" s="102"/>
-      <c r="N34" s="102"/>
-      <c r="O34" s="102"/>
-      <c r="P34" s="102"/>
-      <c r="Q34" s="102"/>
-      <c r="R34" s="102"/>
-      <c r="S34" s="102"/>
-      <c r="T34" s="102"/>
-      <c r="U34" s="102"/>
-      <c r="V34" s="102"/>
-      <c r="W34" s="102"/>
-      <c r="X34" s="102"/>
-      <c r="Y34" s="102"/>
-      <c r="Z34" s="102"/>
-      <c r="AA34" s="102"/>
-      <c r="AB34" s="102"/>
-      <c r="AC34" s="102"/>
-      <c r="AD34" s="102"/>
-      <c r="AE34" s="102"/>
-      <c r="AF34" s="102"/>
-      <c r="AG34" s="103"/>
+      <c r="A34" s="77"/>
+      <c r="B34" s="78"/>
+      <c r="C34" s="78"/>
+      <c r="D34" s="78"/>
+      <c r="E34" s="78"/>
+      <c r="F34" s="79"/>
+      <c r="G34" s="79"/>
+      <c r="H34" s="79"/>
+      <c r="I34" s="79"/>
+      <c r="J34" s="79"/>
+      <c r="K34" s="79"/>
+      <c r="L34" s="79"/>
+      <c r="M34" s="79"/>
+      <c r="N34" s="79"/>
+      <c r="O34" s="79"/>
+      <c r="P34" s="79"/>
+      <c r="Q34" s="79"/>
+      <c r="R34" s="79"/>
+      <c r="S34" s="79"/>
+      <c r="T34" s="79"/>
+      <c r="U34" s="79"/>
+      <c r="V34" s="79"/>
+      <c r="W34" s="79"/>
+      <c r="X34" s="79"/>
+      <c r="Y34" s="79"/>
+      <c r="Z34" s="79"/>
+      <c r="AA34" s="79"/>
+      <c r="AB34" s="79"/>
+      <c r="AC34" s="79"/>
+      <c r="AD34" s="79"/>
+      <c r="AE34" s="79"/>
+      <c r="AF34" s="79"/>
+      <c r="AG34" s="80"/>
     </row>
     <row r="35" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="104"/>
-      <c r="B35" s="102"/>
-      <c r="C35" s="102"/>
-      <c r="D35" s="102"/>
-      <c r="E35" s="102"/>
-      <c r="F35" s="102"/>
-      <c r="G35" s="102"/>
-      <c r="H35" s="102"/>
-      <c r="I35" s="102"/>
-      <c r="J35" s="102"/>
-      <c r="K35" s="102"/>
-      <c r="L35" s="102"/>
-      <c r="M35" s="102"/>
-      <c r="N35" s="102"/>
-      <c r="O35" s="102"/>
-      <c r="P35" s="102"/>
-      <c r="Q35" s="102"/>
-      <c r="R35" s="102"/>
-      <c r="S35" s="102"/>
-      <c r="T35" s="102"/>
-      <c r="U35" s="102"/>
-      <c r="V35" s="102"/>
-      <c r="W35" s="102"/>
-      <c r="X35" s="102"/>
-      <c r="Y35" s="102"/>
-      <c r="Z35" s="102"/>
-      <c r="AA35" s="102"/>
-      <c r="AB35" s="102"/>
-      <c r="AC35" s="102"/>
-      <c r="AD35" s="102"/>
-      <c r="AE35" s="102"/>
-      <c r="AF35" s="102"/>
-      <c r="AG35" s="105"/>
+      <c r="A35" s="81"/>
+      <c r="B35" s="79"/>
+      <c r="C35" s="79"/>
+      <c r="D35" s="79"/>
+      <c r="E35" s="79"/>
+      <c r="F35" s="79"/>
+      <c r="G35" s="79"/>
+      <c r="H35" s="79"/>
+      <c r="I35" s="79"/>
+      <c r="J35" s="79"/>
+      <c r="K35" s="79"/>
+      <c r="L35" s="79"/>
+      <c r="M35" s="79"/>
+      <c r="N35" s="79"/>
+      <c r="O35" s="79"/>
+      <c r="P35" s="79"/>
+      <c r="Q35" s="79"/>
+      <c r="R35" s="79"/>
+      <c r="S35" s="79"/>
+      <c r="T35" s="79"/>
+      <c r="U35" s="79"/>
+      <c r="V35" s="79"/>
+      <c r="W35" s="79"/>
+      <c r="X35" s="79"/>
+      <c r="Y35" s="79"/>
+      <c r="Z35" s="79"/>
+      <c r="AA35" s="79"/>
+      <c r="AB35" s="79"/>
+      <c r="AC35" s="79"/>
+      <c r="AD35" s="79"/>
+      <c r="AE35" s="79"/>
+      <c r="AF35" s="79"/>
+      <c r="AG35" s="82"/>
     </row>
     <row r="36" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="68" t="s">
+      <c r="A36" s="86" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="69"/>
-      <c r="C36" s="69"/>
-      <c r="D36" s="69"/>
-      <c r="E36" s="69"/>
-      <c r="F36" s="69"/>
-      <c r="G36" s="69"/>
-      <c r="H36" s="69"/>
-      <c r="I36" s="69"/>
-      <c r="J36" s="69"/>
-      <c r="K36" s="69"/>
-      <c r="L36" s="69"/>
-      <c r="M36" s="69"/>
-      <c r="N36" s="69"/>
-      <c r="O36" s="69"/>
-      <c r="P36" s="69"/>
-      <c r="Q36" s="69"/>
-      <c r="R36" s="69"/>
-      <c r="S36" s="69"/>
-      <c r="T36" s="69"/>
-      <c r="U36" s="69"/>
-      <c r="V36" s="69"/>
-      <c r="W36" s="69"/>
-      <c r="X36" s="69"/>
-      <c r="Y36" s="69"/>
-      <c r="Z36" s="69"/>
-      <c r="AA36" s="69"/>
-      <c r="AB36" s="69"/>
-      <c r="AC36" s="69"/>
-      <c r="AD36" s="69"/>
-      <c r="AE36" s="69"/>
-      <c r="AF36" s="69"/>
-      <c r="AG36" s="70"/>
+      <c r="B36" s="87"/>
+      <c r="C36" s="87"/>
+      <c r="D36" s="87"/>
+      <c r="E36" s="87"/>
+      <c r="F36" s="87"/>
+      <c r="G36" s="87"/>
+      <c r="H36" s="87"/>
+      <c r="I36" s="87"/>
+      <c r="J36" s="87"/>
+      <c r="K36" s="87"/>
+      <c r="L36" s="87"/>
+      <c r="M36" s="87"/>
+      <c r="N36" s="87"/>
+      <c r="O36" s="87"/>
+      <c r="P36" s="87"/>
+      <c r="Q36" s="87"/>
+      <c r="R36" s="87"/>
+      <c r="S36" s="87"/>
+      <c r="T36" s="87"/>
+      <c r="U36" s="87"/>
+      <c r="V36" s="87"/>
+      <c r="W36" s="87"/>
+      <c r="X36" s="87"/>
+      <c r="Y36" s="87"/>
+      <c r="Z36" s="87"/>
+      <c r="AA36" s="87"/>
+      <c r="AB36" s="87"/>
+      <c r="AC36" s="87"/>
+      <c r="AD36" s="87"/>
+      <c r="AE36" s="87"/>
+      <c r="AF36" s="87"/>
+      <c r="AG36" s="101"/>
     </row>
     <row r="37" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="112" t="s">
+      <c r="A37" s="67" t="s">
         <v>8</v>
       </c>
-      <c r="B37" s="114" t="s">
+      <c r="B37" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="114" t="s">
+      <c r="C37" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="D37" s="114" t="s">
+      <c r="D37" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="116" t="s">
+      <c r="E37" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="F37" s="93" t="s">
+      <c r="F37" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="G37" s="94"/>
-      <c r="H37" s="93" t="s">
+      <c r="G37" s="63"/>
+      <c r="H37" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="I37" s="94"/>
-      <c r="J37" s="93" t="s">
+      <c r="I37" s="63"/>
+      <c r="J37" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="K37" s="94"/>
-      <c r="L37" s="93" t="s">
+      <c r="K37" s="63"/>
+      <c r="L37" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="M37" s="94"/>
-      <c r="N37" s="93" t="s">
+      <c r="M37" s="63"/>
+      <c r="N37" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="O37" s="94"/>
-      <c r="P37" s="93" t="s">
+      <c r="O37" s="63"/>
+      <c r="P37" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="Q37" s="94"/>
-      <c r="R37" s="93" t="s">
+      <c r="Q37" s="63"/>
+      <c r="R37" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="S37" s="94"/>
-      <c r="T37" s="93" t="s">
+      <c r="S37" s="63"/>
+      <c r="T37" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="U37" s="94"/>
-      <c r="V37" s="93" t="s">
+      <c r="U37" s="63"/>
+      <c r="V37" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="W37" s="94"/>
-      <c r="X37" s="93" t="s">
+      <c r="W37" s="63"/>
+      <c r="X37" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="Y37" s="94"/>
-      <c r="Z37" s="93" t="s">
+      <c r="Y37" s="63"/>
+      <c r="Z37" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="AA37" s="94"/>
-      <c r="AB37" s="93" t="s">
+      <c r="AA37" s="63"/>
+      <c r="AB37" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="AC37" s="94"/>
-      <c r="AD37" s="98" t="s">
+      <c r="AC37" s="63"/>
+      <c r="AD37" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="AE37" s="98" t="s">
+      <c r="AE37" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="AF37" s="98" t="s">
+      <c r="AF37" s="75" t="s">
         <v>25</v>
       </c>
-      <c r="AG37" s="106" t="s">
+      <c r="AG37" s="83" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:33" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="113"/>
-      <c r="B38" s="115"/>
-      <c r="C38" s="115"/>
-      <c r="D38" s="115"/>
-      <c r="E38" s="117"/>
+      <c r="A38" s="68"/>
+      <c r="B38" s="70"/>
+      <c r="C38" s="70"/>
+      <c r="D38" s="70"/>
+      <c r="E38" s="72"/>
       <c r="F38" s="13" t="s">
         <v>32</v>
       </c>
@@ -4282,10 +4335,10 @@
       <c r="AC38" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="AD38" s="99"/>
-      <c r="AE38" s="99"/>
-      <c r="AF38" s="99"/>
-      <c r="AG38" s="107"/>
+      <c r="AD38" s="76"/>
+      <c r="AE38" s="76"/>
+      <c r="AF38" s="76"/>
+      <c r="AG38" s="61"/>
     </row>
     <row r="39" spans="1:33" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="49">
@@ -6419,13 +6472,13 @@
       </c>
     </row>
     <row r="55" spans="1:33" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="65" t="s">
+      <c r="A55" s="98" t="s">
         <v>27</v>
       </c>
-      <c r="B55" s="66"/>
-      <c r="C55" s="66"/>
-      <c r="D55" s="66"/>
-      <c r="E55" s="66"/>
+      <c r="B55" s="99"/>
+      <c r="C55" s="99"/>
+      <c r="D55" s="99"/>
+      <c r="E55" s="99"/>
       <c r="F55" s="52" t="e">
         <f>SUM(F39:F54)</f>
         <v>#VALUE!</v>
@@ -6540,41 +6593,41 @@
       </c>
     </row>
     <row r="56" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A56" s="109" t="s">
+      <c r="A56" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="B56" s="109"/>
-      <c r="C56" s="109"/>
-      <c r="D56" s="109"/>
-      <c r="E56" s="109"/>
-      <c r="F56" s="109"/>
-      <c r="G56" s="109"/>
-      <c r="H56" s="109"/>
-      <c r="I56" s="109"/>
-      <c r="J56" s="109"/>
-      <c r="K56" s="109"/>
-      <c r="L56" s="109"/>
-      <c r="M56" s="109"/>
-      <c r="N56" s="109"/>
-      <c r="O56" s="109"/>
-      <c r="P56" s="109"/>
-      <c r="Q56" s="109"/>
-      <c r="R56" s="109"/>
-      <c r="S56" s="109"/>
-      <c r="T56" s="109"/>
-      <c r="U56" s="109"/>
-      <c r="V56" s="109"/>
-      <c r="W56" s="109"/>
-      <c r="X56" s="109"/>
-      <c r="Y56" s="109"/>
-      <c r="Z56" s="109"/>
-      <c r="AA56" s="109"/>
-      <c r="AB56" s="109"/>
-      <c r="AC56" s="109"/>
-      <c r="AD56" s="109"/>
-      <c r="AE56" s="109"/>
-      <c r="AF56" s="109"/>
-      <c r="AG56" s="109"/>
+      <c r="B56" s="64"/>
+      <c r="C56" s="64"/>
+      <c r="D56" s="64"/>
+      <c r="E56" s="64"/>
+      <c r="F56" s="64"/>
+      <c r="G56" s="64"/>
+      <c r="H56" s="64"/>
+      <c r="I56" s="64"/>
+      <c r="J56" s="64"/>
+      <c r="K56" s="64"/>
+      <c r="L56" s="64"/>
+      <c r="M56" s="64"/>
+      <c r="N56" s="64"/>
+      <c r="O56" s="64"/>
+      <c r="P56" s="64"/>
+      <c r="Q56" s="64"/>
+      <c r="R56" s="64"/>
+      <c r="S56" s="64"/>
+      <c r="T56" s="64"/>
+      <c r="U56" s="64"/>
+      <c r="V56" s="64"/>
+      <c r="W56" s="64"/>
+      <c r="X56" s="64"/>
+      <c r="Y56" s="64"/>
+      <c r="Z56" s="64"/>
+      <c r="AA56" s="64"/>
+      <c r="AB56" s="64"/>
+      <c r="AC56" s="64"/>
+      <c r="AD56" s="64"/>
+      <c r="AE56" s="64"/>
+      <c r="AF56" s="64"/>
+      <c r="AG56" s="64"/>
     </row>
     <row r="57" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="58" spans="1:33" ht="18" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -6624,8 +6677,56 @@
     <row r="102" ht="18" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="103" ht="18" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="o8ACUjwZ60BmxDGubwQ0f2wgb3nM2ipXUlNJ5p3kVSJlpm38TkYhGQuqkIKY0LhXcF5pV6bApbwh+jb1w4P98A==" saltValue="fFusfQ3GfE0183oXy/pf3w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Wob0+sEsSpo4TIxI4d9NMp/zKFxo8MCQv+pnjQOWmrT0bhcLeuysZRoIcIeYhKFvp2Px1+WKJdqwMRFTBKOPew==" saltValue="WeckCvwxyAVdZ0JfTQGDjg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="64">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="H2:AC13"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="H1:AC1"/>
+    <mergeCell ref="A36:AG36"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A15:AG15"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="V16:W16"/>
+    <mergeCell ref="X16:Y16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="A14:AG14"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="AD16:AD17"/>
+    <mergeCell ref="AE16:AE17"/>
+    <mergeCell ref="AF16:AF17"/>
+    <mergeCell ref="A34:AG35"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="P37:Q37"/>
+    <mergeCell ref="R37:S37"/>
+    <mergeCell ref="T37:U37"/>
+    <mergeCell ref="V37:W37"/>
+    <mergeCell ref="X37:Y37"/>
+    <mergeCell ref="Z37:AA37"/>
+    <mergeCell ref="AB37:AC37"/>
+    <mergeCell ref="AE37:AE38"/>
+    <mergeCell ref="AF37:AF38"/>
+    <mergeCell ref="AG37:AG38"/>
     <mergeCell ref="AG16:AG17"/>
     <mergeCell ref="Z16:AA16"/>
     <mergeCell ref="AB16:AC16"/>
@@ -6642,54 +6743,6 @@
     <mergeCell ref="D16:D17"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="AD37:AD38"/>
-    <mergeCell ref="A34:AG35"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="P37:Q37"/>
-    <mergeCell ref="R37:S37"/>
-    <mergeCell ref="T37:U37"/>
-    <mergeCell ref="V37:W37"/>
-    <mergeCell ref="X37:Y37"/>
-    <mergeCell ref="Z37:AA37"/>
-    <mergeCell ref="AB37:AC37"/>
-    <mergeCell ref="AE37:AE38"/>
-    <mergeCell ref="AF37:AF38"/>
-    <mergeCell ref="AG37:AG38"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A15:AG15"/>
-    <mergeCell ref="T16:U16"/>
-    <mergeCell ref="V16:W16"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="A14:AG14"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="AD16:AD17"/>
-    <mergeCell ref="AE16:AE17"/>
-    <mergeCell ref="AF16:AF17"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="H2:AC13"/>
-    <mergeCell ref="A55:E55"/>
-    <mergeCell ref="H1:AC1"/>
-    <mergeCell ref="A36:AG36"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="A33:E33"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="G33">

</xml_diff>